<commit_message>
Polish opening guidance and first retreat recovery hints
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/unlock.xlsx
+++ b/space-battleship/config_excel/unlock.xlsx
@@ -1324,7 +1324,7 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>装备已自动装载，可在下方直接升级。</t>
+          <t>左下生命条来自装甲。试着升一级装甲，再看看防御卡和生命上限的变化。</t>
         </is>
       </c>
     </row>
@@ -1359,7 +1359,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>偏转护盾可以抵御能量武器,并且一段时间不受攻击后即能自动恢复</t>
+          <t>在可换装的防御位选「偏转护盾」，看看左下多出的护盾条。避开攻击一段时间后，它会自己恢复。</t>
         </is>
       </c>
     </row>
@@ -1394,7 +1394,7 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>装备已自动装载，可在下方直接升级。</t>
+          <t>战舰已装好一门脉冲激光。给空武器位再装一门，看看舰上多出的炮口；装配免费。</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>我们的科学家研发了导弹,导弹可以同时打击多个敌人,并且当然,能偏转能量的偏转护盾对它效果并不大</t>
+          <t>试着把一个武器位换成追踪导弹。它会追着目标飞；换装免费，这个位置的等级也会保留。</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>谁会喜欢软绵绵的光束?用轰鸣的大炮将对面射成筛子吧.磁轨火炮将洞穿你的敌人,尤其是那些觉得能躲在护盾后面一辈子的软蛋!</t>
+          <t>点一个武器名称，换成磁轨火炮，看看它发射时贯穿战场的亮线。换装免费，等级保留。</t>
         </is>
       </c>
     </row>
@@ -1709,7 +1709,7 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>我们调查这些..铀?得到了一些东西.利用它可以生产大量能量,然后增强我们的所有系统.不过要注意,往同一个系统注入过多能量,会使得能量不稳定,我们将额外分配一些能量用于维持系统,这会导致能量的效果降低.</t>
+          <t>打开「反应炉」，先点「均分」分配能源，看看右侧加成亮起来。想增强某一项，再拖动对应能源条。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: integrate action-led guidance, earned help and first-defeat safeguards
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/unlock.xlsx
+++ b/space-battleship/config_excel/unlock.xlsx
@@ -1324,7 +1324,7 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>装备已自动装载，可在下方直接升级。</t>
+          <t>左下生命条来自装甲。试着升一级装甲，再看看防御卡和生命上限的变化。</t>
         </is>
       </c>
     </row>
@@ -1359,7 +1359,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>偏转护盾可以抵御能量武器,并且一段时间不受攻击后即能自动恢复</t>
+          <t>在可换装的防御位选「偏转护盾」，看看左下多出的护盾条。避开攻击一段时间后，它会自己恢复。</t>
         </is>
       </c>
     </row>
@@ -1394,7 +1394,7 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>装备已自动装载，可在下方直接升级。</t>
+          <t>战舰已装好一门脉冲激光。给空武器位再装一门，看看舰上多出的炮口；装配免费。</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>我们的科学家研发了导弹,导弹可以同时打击多个敌人,并且当然,能偏转能量的偏转护盾对它效果并不大</t>
+          <t>试着把一个武器位换成追踪导弹。它会追着目标飞；换装免费，这个位置的等级也会保留。</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>谁会喜欢软绵绵的光束?用轰鸣的大炮将对面射成筛子吧.磁轨火炮将洞穿你的敌人,尤其是那些觉得能躲在护盾后面一辈子的软蛋!</t>
+          <t>点一个武器名称，换成磁轨火炮，看看它发射时贯穿战场的亮线。换装免费，等级保留。</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>第6关会遇到持续恢复护盾的敌舰。光束保持锁定时伤害逐渐增强，可突破恢复；短促攻击可能被恢复抵消。</t>
+          <t>先把一门武器换成光束，看看同一艘敌舰的护盾能否被压住。光束持续照射才会增伤；若还打不穿，先升级这门武器再试。</t>
         </is>
       </c>
     </row>
@@ -1762,7 +1762,7 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>哦对对对,看看这个新玩意,AI工厂!这些不知疲倦的劳工将解决我们的资源生产问题..当然,我知道,资源的需求是永无止境的...</t>
+          <t>打开「AI工厂」，先「生成×1」，再给炼铁炉分配「+1 AI」。看看施工开始；建好后，它会定时产出铁。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Teach cannon cadence through a first refit experiment
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/unlock.xlsx
+++ b/space-battleship/config_excel/unlock.xlsx
@@ -1464,7 +1464,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>点一个武器名称，换成磁轨火炮，看看它发射时贯穿战场的亮线。换装免费，等级保留。</t>
+          <t>换一门磁轨火炮，看看它一发打掉多少血，再看下一发要等多久。换装免费，等级保留。</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>先把一门武器换成光束，看看同一艘敌舰的护盾能否被压住。光束持续照射才会增伤；若还打不穿，先升级这门武器再试。</t>
+          <t>先把一门武器换成光束，看看同一艘敌舰的血条是否降得越来越快。光束持续照射才会增伤；若打不动，指向敌舰查看防御，再试另一类伤害。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reconcile tutorial workbook with integrated reactor and planet text
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/unlock.xlsx
+++ b/space-battleship/config_excel/unlock.xlsx
@@ -1709,7 +1709,7 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>打开「反应炉」，先点「均分」分配能源，看看右侧加成亮起来。想增强某一项，再拖动对应能源条。</t>
+          <t>反应炉已接通。去「反应炉」点「均分」，看看各模块的加成；也可以拖动能量条，把更多能源分给想加强的模块。</t>
         </is>
       </c>
     </row>
@@ -2147,7 +2147,7 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>通关30后可派遣空闲船员探索首颗星球。探索中建设新型船坞，并派入建筑要求的额外船员；建成后领取设施，开启重铸。重铸保留铁与铀余额与永久探索奖励，重置本轮养成，从第5关再出发。</t>
+          <t>去「星球探索」，派一名空闲船员出发。完成一次探索后，看看探索度和星球加成的变化；设施可用时，点设施继续建设。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Point earned hull and first crew tutorials to their next playable action
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/unlock.xlsx
+++ b/space-battleship/config_excel/unlock.xlsx
@@ -1569,7 +1569,7 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>当然,我们的科学家研发了新的战舰,你可以立即试试了...撕碎你的敌人吧</t>
+          <t>到「战舰」启用飞燕护卫舰，再点新增W04空槽免费装武器，看它随舰开火。</t>
         </is>
       </c>
     </row>
@@ -1937,7 +1937,7 @@
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>嗯,也许你需要一些真人来陪你,我们解冻了一名优秀的船员,你就好好利用他吧</t>
+          <t>去「船员」先看岗位的自动花费预告，再确认分配；想停就点「解除分配」。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
work: integrate crew confirmation and first-use clarity candidates
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/unlock.xlsx
+++ b/space-battleship/config_excel/unlock.xlsx
@@ -1569,7 +1569,7 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>当然,我们的科学家研发了新的战舰,你可以立即试试了...撕碎你的敌人吧</t>
+          <t>到「战舰」启用飞燕护卫舰，再点新增W04空槽免费装武器，看它随舰开火。</t>
         </is>
       </c>
     </row>
@@ -1937,7 +1937,7 @@
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>嗯,也许你需要一些真人来陪你,我们解冻了一名优秀的船员,你就好好利用他吧</t>
+          <t>去「船员」看看岗位会做什么、会花什么，再决定分配；随时可解除分配。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
guide: clarify opening equipment and type matchups
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/unlock.xlsx
+++ b/space-battleship/config_excel/unlock.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="29868" windowHeight="13380" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="unlock" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="unlock" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1359,7 +1359,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>在可换装的防御位选「偏转护盾」，看看左下多出的护盾条。避开攻击一段时间后，它会自己恢复。</t>
+          <t>在防御位免费换入偏转护盾，看左下独立护盾条。它先承受攻击；受击会重置2秒恢复等待。</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>试着把一个武器位换成追踪导弹。它会追着目标飞；换装免费，这个位置的等级也会保留。</t>
+          <t>追踪导弹一次发出多枚物理弹，适合第2关蜂群。选武器位免费换入；槽位等级保留。</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>换一门磁轨火炮，看看它一发打掉多少血，再看下一发要等多久。换装免费，等级保留。</t>
+          <t>磁轨火炮是物理大击，适合单个厚敌，也可试打抗能量护盾；比较单发伤害与下次开火间隔。换装免费，等级保留。</t>
         </is>
       </c>
     </row>
@@ -1709,7 +1709,7 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>反应炉已接通。去「反应炉」点「均分」，看看各模块的加成；也可以拖动能量条，把更多能源分给想加强的模块。</t>
+          <t>反应炉已接通。去「反应炉」点「均分」先看加成，再将能源偏向武器或防御，比较清敌速度与承伤。分配不花铁。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix tutorial and native presentation blockers; propose stage three enemy diff
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/unlock.xlsx
+++ b/space-battleship/config_excel/unlock.xlsx
@@ -1359,7 +1359,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>在防御位免费换入偏转护盾，看左下独立护盾条。它先承受攻击；受击会重置2秒恢复等待。</t>
+          <t>防御位只能装一件：换入偏转护盾会替下复合装甲。护盾偏重抵御能量攻击；受击后等待2秒才恢复。装甲偏重抵御物理攻击。</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>追踪导弹一次发出多枚物理弹，适合第2关蜂群。选武器位免费换入；槽位等级保留。</t>
+          <t>追踪导弹一次发射多枚物理弹，可同时追踪多个目标。选武器位免费换入；槽位等级保留。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tighten tutorial and unlock flow; stop AI research per level
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/unlock.xlsx
+++ b/space-battleship/config_excel/unlock.xlsx
@@ -1324,7 +1324,7 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>左下生命条来自装甲。试着升一级装甲，再看看防御卡和生命上限的变化。</t>
+          <t>复合装甲已解锁。</t>
         </is>
       </c>
     </row>
@@ -1359,7 +1359,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>防御位只能装一件：换入偏转护盾会替下复合装甲。护盾偏重抵御能量攻击；受击后等待2秒才恢复。装甲偏重抵御物理攻击。</t>
+          <t>偏转护盾已解锁。</t>
         </is>
       </c>
     </row>
@@ -1394,7 +1394,7 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>战舰已装好一门脉冲激光。给空武器位再装一门，看看舰上多出的炮口；装配免费。</t>
+          <t>脉冲激光已解锁。</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>追踪导弹一次发射多枚物理弹，可同时追踪多个目标。选武器位免费换入；槽位等级保留。</t>
+          <t>追踪导弹已解锁。</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>磁轨火炮是物理大击，适合单个厚敌，也可试打抗能量护盾；比较单发伤害与下次开火间隔。换装免费，等级保留。</t>
+          <t>磁轨火炮已解锁。</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>先把一门武器换成光束，看看同一艘敌舰的血条是否降得越来越快。光束持续照射才会增伤；若打不动，指向敌舰查看防御，再试另一类伤害。</t>
+          <t>持续锁定光束已解锁。</t>
         </is>
       </c>
     </row>
@@ -1534,7 +1534,7 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>可在战舰页面启用游隼侦察艇。</t>
+          <t>游隼侦察艇已解锁。</t>
         </is>
       </c>
     </row>
@@ -1569,7 +1569,7 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>到「战舰」启用飞燕护卫舰，再点新增W04空槽免费装武器，看它随舰开火。</t>
+          <t>飞燕护卫舰已解锁。</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>这艘船,很大,很强,很暴力,他有更多的武器,来帮助你干掉所有对手</t>
+          <t>云鳐巡洋舰已解锁。</t>
         </is>
       </c>
     </row>
@@ -1639,7 +1639,7 @@
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>这是我们能提供的最强的战舰了,相信我,它能陪你走到最后</t>
+          <t>玄甲战列舰已解锁。</t>
         </is>
       </c>
     </row>
@@ -1674,7 +1674,7 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>我之前说过那是我们能提供的最强战舰了吗?有了新船坞,那已经是过去式了,这艘新船将更有力的摧毁你的敌人.</t>
+          <t>白鲸无畏舰已解锁。</t>
         </is>
       </c>
     </row>
@@ -1709,7 +1709,7 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>反应炉已接通。去「反应炉」点「均分」先看加成，再将能源偏向武器或防御，比较清敌速度与承伤。分配不花铁。</t>
+          <t>反应炉已解锁。</t>
         </is>
       </c>
     </row>
@@ -1762,7 +1762,7 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>打开「AI工厂」，先「生成×1」，再给炼铁炉分配「+1 AI」。看看施工开始；建好后，它会定时产出铁。</t>
+          <t>超时空炼铁炉已解锁。</t>
         </is>
       </c>
     </row>
@@ -1797,7 +1797,7 @@
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>通过这个全新的工厂产物,我们让武器的效率有了进一步提升,感谢AI吧,它们什么都不需要,只要..你给一些能源</t>
+          <t>正电子聚焦装置已解锁。</t>
         </is>
       </c>
     </row>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>这是调查致密恒星的构造后得出的结论,而我们的无休劳动者正在不断的生产这种全宇宙最硬的物质.它将提升我们的所有防御能力..船体,护盾,当然,你变得更耐打了!</t>
+          <t>简并态装甲已解锁。</t>
         </is>
       </c>
     </row>
@@ -1867,7 +1867,7 @@
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>这下我们终于有办法进一步从无用的残骸里回收更多的强化碎片了,真是非常感谢!</t>
+          <t>强化碎片熔炼炉已解锁。</t>
         </is>
       </c>
     </row>
@@ -1902,7 +1902,7 @@
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>敌舰残骸中可回收强化碎片，用于提升全局装备强化等级。</t>
+          <t>装备强化已解锁。</t>
         </is>
       </c>
     </row>
@@ -1937,7 +1937,7 @@
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>去「船员」看看岗位会做什么、会花什么，再决定分配；随时可解除分配。</t>
+          <t>船员01已解锁。</t>
         </is>
       </c>
     </row>
@@ -1972,7 +1972,7 @@
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>已解锁船员02，可在船员页分配到游戏系统。</t>
+          <t>船员02已解锁。</t>
         </is>
       </c>
     </row>
@@ -2007,7 +2007,7 @@
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>已解锁船员03，可在船员页分配到游戏系统。</t>
+          <t>船员03已解锁。</t>
         </is>
       </c>
     </row>
@@ -2042,7 +2042,7 @@
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>已解锁船员04，可在船员页分配到游戏系统。</t>
+          <t>船员04已解锁。</t>
         </is>
       </c>
     </row>
@@ -2077,7 +2077,7 @@
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>已解锁船员05，可在船员页分配到游戏系统。</t>
+          <t>船员05已解锁。</t>
         </is>
       </c>
     </row>
@@ -2112,7 +2112,7 @@
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>已解锁船员06，可在船员页分配到游戏系统。</t>
+          <t>船员06已解锁。</t>
         </is>
       </c>
     </row>
@@ -2147,7 +2147,7 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>去「星球探索」，派一名空闲船员出发。完成一次探索后，看看探索度和星球加成的变化；设施可用时，点设施继续建设。</t>
+          <t>星球探索已解锁。</t>
         </is>
       </c>
     </row>
@@ -2182,7 +2182,7 @@
       </c>
       <c r="G30" s="0" t="inlineStr">
         <is>
-          <t>船员可以获得经验并提升等级。</t>
+          <t>船员等级已解锁。</t>
         </is>
       </c>
     </row>
@@ -2217,7 +2217,7 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>反应炉充能可以提升强化碎片产出，让装备强化继续成长。</t>
+          <t>强化凝聚已解锁。</t>
         </is>
       </c>
     </row>
@@ -2252,7 +2252,7 @@
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>已发现该星系的气态行星,可以进一步探索该行星系</t>
+          <t>新行星已发现。</t>
         </is>
       </c>
     </row>
@@ -2287,7 +2287,7 @@
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>已准备好探索该星系</t>
+          <t>新行星已发现。</t>
         </is>
       </c>
     </row>
@@ -2322,7 +2322,7 @@
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>哦,一个生命末期的恒星,它能给我们什么?</t>
+          <t>新行星已发现。</t>
         </is>
       </c>
     </row>
@@ -2357,7 +2357,7 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>恒星的残骸...但仍旧蕴含让我们需要的资源..</t>
+          <t>新行星已发现。</t>
         </is>
       </c>
     </row>
@@ -2392,7 +2392,7 @@
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>这颗死亡的恒星释放出强大的能量,我们需要控制它</t>
+          <t>新行星已发现。</t>
         </is>
       </c>
     </row>
@@ -2427,7 +2427,7 @@
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>现在我们可以殖民星系了,快派遣船员出发吧</t>
+          <t>星系殖民已解锁。</t>
         </is>
       </c>
     </row>
@@ -2462,7 +2462,7 @@
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t>已解锁船员07，可在船员页分配到游戏系统。</t>
+          <t>船员07已解锁。</t>
         </is>
       </c>
     </row>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="G39" s="0" t="inlineStr">
         <is>
-          <t>已解锁船员08，可在船员页分配到游戏系统。</t>
+          <t>船员08已解锁。</t>
         </is>
       </c>
     </row>
@@ -2532,7 +2532,7 @@
       </c>
       <c r="G40" s="0" t="inlineStr">
         <is>
-          <t>已解锁船员09，可在船员页分配到游戏系统。</t>
+          <t>船员09已解锁。</t>
         </is>
       </c>
     </row>
@@ -2567,7 +2567,7 @@
       </c>
       <c r="G41" s="0" t="inlineStr">
         <is>
-          <t>已解锁船员10，可在船员页分配到游戏系统。</t>
+          <t>船员10已解锁。</t>
         </is>
       </c>
     </row>
@@ -2602,7 +2602,7 @@
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>已解锁船员11，可在船员页分配到游戏系统。</t>
+          <t>船员11已解锁。</t>
         </is>
       </c>
     </row>
@@ -2637,7 +2637,7 @@
       </c>
       <c r="G43" s="0" t="inlineStr">
         <is>
-          <t>已解锁船员12，可在船员页分配到游戏系统。</t>
+          <t>船员12已解锁。</t>
         </is>
       </c>
     </row>
@@ -2672,7 +2672,7 @@
       </c>
       <c r="G44" s="0" t="inlineStr">
         <is>
-          <t>已解锁船员13，可在船员页分配到游戏系统。</t>
+          <t>船员13已解锁。</t>
         </is>
       </c>
     </row>
@@ -2707,7 +2707,7 @@
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>已解锁船员14，可在船员页分配到游戏系统。</t>
+          <t>船员14已解锁。</t>
         </is>
       </c>
     </row>
@@ -2742,7 +2742,7 @@
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>已解锁船员15，可在船员页分配到游戏系统。</t>
+          <t>船员15已解锁。</t>
         </is>
       </c>
     </row>
@@ -2777,7 +2777,7 @@
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>已解锁船员16，可在船员页分配到游戏系统。</t>
+          <t>船员16已解锁。</t>
         </is>
       </c>
     </row>
@@ -2812,7 +2812,7 @@
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>已解锁船员17，可在船员页分配到游戏系统。</t>
+          <t>船员17已解锁。</t>
         </is>
       </c>
     </row>
@@ -2847,7 +2847,7 @@
       </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
-          <t>已解锁船员18，可在船员页分配到游戏系统。</t>
+          <t>船员18已解锁。</t>
         </is>
       </c>
     </row>
@@ -2882,7 +2882,7 @@
       </c>
       <c r="G50" s="0" t="inlineStr">
         <is>
-          <t>已解锁船员19，可在船员页分配到游戏系统。</t>
+          <t>船员19已解锁。</t>
         </is>
       </c>
     </row>
@@ -2917,7 +2917,7 @@
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>已解锁船员20，可在船员页分配到游戏系统。</t>
+          <t>船员20已解锁。</t>
         </is>
       </c>
     </row>

</xml_diff>